<commit_message>
feat(web): improve PWA navigation and install experience
</commit_message>
<xml_diff>
--- a/data/subadapp.xlsx
+++ b/data/subadapp.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" dateCompatibility="false"/>
+  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="291" uniqueCount="228">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="291" uniqueCount="234">
   <si>
     <t xml:space="preserve">no</t>
   </si>
@@ -107,7 +107,7 @@
     <t xml:space="preserve">https://ansiklopedi.subadapcocuk.org/index.php/Kabuk_Kırma_Partisi_(2024)</t>
   </si>
   <si>
-    <t xml:space="preserve">https://ansiklopedi.subadapcocuk.org/index.php/Dosya:Kabuk_k%C4%B1rma_partisi_alb%C3%BCm_kapa%C4%9F%C4%B1.png</t>
+    <t xml:space="preserve">https://ansiklopedi.subadapcocuk.org/images/thumb/5/59/Kabuk_k%C4%B1rma_partisi_alb%C3%BCm_kapa%C4%9F%C4%B1.png/300px-Kabuk_k%C4%B1rma_partisi_alb%C3%BCm_kapa%C4%9F%C4%B1.png</t>
   </si>
   <si>
     <t xml:space="preserve">albumNo</t>
@@ -662,6 +662,9 @@
     <t xml:space="preserve">https://ansiklopedi.subadapcocuk.org/images/3/31/Suzi.mp3</t>
   </si>
   <si>
+    <t xml:space="preserve">https://ansiklopedi.subadapcocuk.org/images/thumb/3/3e/SUZ%C4%B0.png/300px-SUZ%C4%B0.png</t>
+  </si>
+  <si>
     <t xml:space="preserve">Tak Tak Tak</t>
   </si>
   <si>
@@ -671,6 +674,9 @@
     <t xml:space="preserve">https://ansiklopedi.subadapcocuk.org/images/9/96/Tak_Tak_Tak.mp3</t>
   </si>
   <si>
+    <t xml:space="preserve">https://ansiklopedi.subadapcocuk.org/images/thumb/8/80/TAK_TAK_TAK.png/300px-TAK_TAK_TAK.png</t>
+  </si>
+  <si>
     <t xml:space="preserve">Şaşıran Mevsimler</t>
   </si>
   <si>
@@ -680,6 +686,9 @@
     <t xml:space="preserve">https://ansiklopedi.subadapcocuk.org/images/c/c4/%C5%9Ea%C5%9F%C4%B1ran_Mevsimler.mp3</t>
   </si>
   <si>
+    <t xml:space="preserve">https://ansiklopedi.subadapcocuk.org/images/thumb/1/16/MEVS%C4%B0MLER.png/300px-MEVS%C4%B0MLER.png</t>
+  </si>
+  <si>
     <t xml:space="preserve">Evdeki Hayalet</t>
   </si>
   <si>
@@ -689,6 +698,9 @@
     <t xml:space="preserve">https://ansiklopedi.subadapcocuk.org/images/0/0b/Evdeki_Hayalet.mp3</t>
   </si>
   <si>
+    <t xml:space="preserve">https://ansiklopedi.subadapcocuk.org/images/thumb/e/e5/EVDEK%C4%B0_HAYALET.png/300px-EVDEK%C4%B0_HAYALET.png</t>
+  </si>
+  <si>
     <t xml:space="preserve">Takıl Kitapların Kanatlarına</t>
   </si>
   <si>
@@ -698,6 +710,9 @@
     <t xml:space="preserve">https://ansiklopedi.subadapcocuk.org/images/f/f8/Tak%C4%B1l_Kitaplar%C4%B1n_Kanatlar%C4%B1na.mp3</t>
   </si>
   <si>
+    <t xml:space="preserve">https://ansiklopedi.subadapcocuk.org/images/thumb/2/26/TAKIL_K%C4%B0TAPLARIN_KANATLARINA.png/300px-TAKIL_K%C4%B0TAPLARIN_KANATLARINA.png</t>
+  </si>
+  <si>
     <t xml:space="preserve">Öcü Möcü Yok Ki! </t>
   </si>
   <si>
@@ -705,6 +720,9 @@
   </si>
   <si>
     <t xml:space="preserve">https://ansiklopedi.subadapcocuk.org/images/9/9a/%C3%96c%C3%BC_M%C3%B6c%C3%BC_Yok_Ki.mp3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://ansiklopedi.subadapcocuk.org/images/thumb/5/5d/%C3%96c%C3%BC_m%C3%B6c%C3%BC_yom_ki.png/300px-%C3%96c%C3%BC_m%C3%B6c%C3%BC_yom_ki.png</t>
   </si>
 </sst>
 </file>
@@ -755,19 +773,21 @@
     <font>
       <sz val="10"/>
       <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF0000FF"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Times New Roman"/>
       <family val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF0000FF"/>
-      <name val="Arial"/>
-      <family val="2"/>
       <charset val="1"/>
     </font>
   </fonts>
@@ -844,7 +864,7 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
@@ -852,7 +872,7 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -936,37 +956,37 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="44546a"/>
+        <a:srgbClr val="44546A"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="e7e6e6"/>
+        <a:srgbClr val="E7E6E6"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4472c4"/>
+        <a:srgbClr val="4472C4"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="ed7d31"/>
+        <a:srgbClr val="ED7D31"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="a5a5a5"/>
+        <a:srgbClr val="A5A5A5"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="ffc000"/>
+        <a:srgbClr val="FFC000"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="5b9bd5"/>
+        <a:srgbClr val="5B9BD5"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="70ad47"/>
+        <a:srgbClr val="70AD47"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0563c1"/>
+        <a:srgbClr val="0563C1"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="954f72"/>
+        <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
@@ -1264,20 +1284,11 @@
       <c r="D9" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="E9" s="5" t="s">
         <v>28</v>
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="E4" r:id="rId1" display="http://ansiklopedi.subadapcocuk.org/images/thumb/3/3c/Kapak_anasayfa.png/300px-Kapak_anasayfa.png"/>
-    <hyperlink ref="D6" r:id="rId2" display="http://ansiklopedi.subadapcocuk.org/index.php/Hayal_Et_(2019)"/>
-    <hyperlink ref="E6" r:id="rId3" display="https://ansiklopedi.subadapcocuk.org/images/thumb/3/34/Hayal-Et-alb%C3%BCm-g%C3%B6rseli-O%C4%9Fuz-Demir-1024x1024.jpg/300px-Hayal-Et-alb%C3%BCm-g%C3%B6rseli-O%C4%9Fuz-Demir-1024x1024.jpg"/>
-    <hyperlink ref="D7" r:id="rId4" display="http://ansiklopedi.subadapcocuk.org/index.php/Hey,_Buraya_Baksan%C4%B1za!_(2020)"/>
-    <hyperlink ref="D8" r:id="rId5" display="https://ansiklopedi.subadapcocuk.org/index.php/Birimiz_Hepimiz_-_Hepimiz_Birimiz_(2023)"/>
-    <hyperlink ref="E8" r:id="rId6" display="https://ansiklopedi.subadapcocuk.org/images/thumb/5/5b/Kapak.jpg/300px-Kapak.jpg"/>
-    <hyperlink ref="D9" r:id="rId7" display="https://ansiklopedi.subadapcocuk.org/index.php/Kabuk_Kırma_Partisi_(2024)"/>
-  </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -1335,7 +1346,7 @@
       <c r="B2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" s="6" t="s">
         <v>5</v>
       </c>
       <c r="D2" s="2" t="s">
@@ -1358,7 +1369,7 @@
       <c r="B3" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="2" t="s">
         <v>5</v>
       </c>
       <c r="D3" s="2" t="s">
@@ -1381,7 +1392,7 @@
       <c r="B4" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="6" t="s">
         <v>5</v>
       </c>
       <c r="D4" s="2" t="s">
@@ -1404,7 +1415,7 @@
       <c r="B5" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="6" t="s">
         <v>5</v>
       </c>
       <c r="D5" s="2" t="s">
@@ -1427,7 +1438,7 @@
       <c r="B6" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="6" t="s">
         <v>5</v>
       </c>
       <c r="D6" s="2" t="s">
@@ -1450,7 +1461,7 @@
       <c r="B7" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" s="6" t="s">
         <v>5</v>
       </c>
       <c r="D7" s="2" t="s">
@@ -1473,7 +1484,7 @@
       <c r="B8" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="C8" s="7" t="s">
         <v>56</v>
       </c>
       <c r="D8" s="2" t="s">
@@ -1496,7 +1507,7 @@
       <c r="B9" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="C9" s="7" t="s">
         <v>56</v>
       </c>
       <c r="D9" s="2" t="s">
@@ -1519,7 +1530,7 @@
       <c r="B10" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="C10" s="6" t="s">
+      <c r="C10" s="7" t="s">
         <v>56</v>
       </c>
       <c r="D10" s="2" t="s">
@@ -1542,7 +1553,7 @@
       <c r="B11" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="C11" s="7" t="s">
         <v>56</v>
       </c>
       <c r="D11" s="2" t="s">
@@ -1565,7 +1576,7 @@
       <c r="B12" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="C12" s="6" t="s">
+      <c r="C12" s="7" t="s">
         <v>56</v>
       </c>
       <c r="D12" s="2" t="s">
@@ -1588,7 +1599,7 @@
       <c r="B13" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="C13" s="6" t="s">
+      <c r="C13" s="7" t="s">
         <v>56</v>
       </c>
       <c r="D13" s="2" t="s">
@@ -2376,14 +2387,14 @@
       <c r="D47" s="2" t="s">
         <v>210</v>
       </c>
-      <c r="E47" s="7" t="s">
+      <c r="E47" s="5" t="s">
         <v>211</v>
       </c>
-      <c r="F47" s="7" t="s">
+      <c r="F47" s="5" t="s">
         <v>212</v>
       </c>
-      <c r="G47" s="7" t="s">
-        <v>28</v>
+      <c r="G47" s="5" t="s">
+        <v>213</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2397,16 +2408,16 @@
         <v>26</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>213</v>
-      </c>
-      <c r="E48" s="7" t="s">
         <v>214</v>
       </c>
-      <c r="F48" s="7" t="s">
+      <c r="E48" s="5" t="s">
         <v>215</v>
       </c>
-      <c r="G48" s="7" t="s">
-        <v>28</v>
+      <c r="F48" s="5" t="s">
+        <v>216</v>
+      </c>
+      <c r="G48" s="5" t="s">
+        <v>217</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2420,16 +2431,16 @@
         <v>26</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>216</v>
-      </c>
-      <c r="E49" s="7" t="s">
-        <v>217</v>
-      </c>
-      <c r="F49" s="7" t="s">
         <v>218</v>
       </c>
-      <c r="G49" s="7" t="s">
-        <v>28</v>
+      <c r="E49" s="5" t="s">
+        <v>219</v>
+      </c>
+      <c r="F49" s="5" t="s">
+        <v>220</v>
+      </c>
+      <c r="G49" s="5" t="s">
+        <v>221</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2443,16 +2454,16 @@
         <v>26</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>219</v>
-      </c>
-      <c r="E50" s="7" t="s">
-        <v>220</v>
-      </c>
-      <c r="F50" s="7" t="s">
-        <v>221</v>
-      </c>
-      <c r="G50" s="7" t="s">
-        <v>28</v>
+        <v>222</v>
+      </c>
+      <c r="E50" s="5" t="s">
+        <v>223</v>
+      </c>
+      <c r="F50" s="5" t="s">
+        <v>224</v>
+      </c>
+      <c r="G50" s="5" t="s">
+        <v>225</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2466,16 +2477,16 @@
         <v>26</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>222</v>
-      </c>
-      <c r="E51" s="7" t="s">
-        <v>223</v>
-      </c>
-      <c r="F51" s="7" t="s">
-        <v>224</v>
-      </c>
-      <c r="G51" s="7" t="s">
-        <v>28</v>
+        <v>226</v>
+      </c>
+      <c r="E51" s="5" t="s">
+        <v>227</v>
+      </c>
+      <c r="F51" s="5" t="s">
+        <v>228</v>
+      </c>
+      <c r="G51" s="5" t="s">
+        <v>229</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2489,61 +2500,19 @@
         <v>26</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>225</v>
-      </c>
-      <c r="E52" s="7" t="s">
-        <v>226</v>
-      </c>
-      <c r="F52" s="7" t="s">
-        <v>227</v>
-      </c>
-      <c r="G52" s="7" t="s">
-        <v>28</v>
+        <v>230</v>
+      </c>
+      <c r="E52" s="5" t="s">
+        <v>231</v>
+      </c>
+      <c r="F52" s="5" t="s">
+        <v>232</v>
+      </c>
+      <c r="G52" s="5" t="s">
+        <v>233</v>
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="C2" r:id="rId1" display="Bilmiş Çocuğun Şarkıları"/>
-    <hyperlink ref="G2" r:id="rId2" display="https://ansiklopedi.subadapcocuk.org/images/thumb/e/e9/D%C3%BC%C5%9F-r.png/300px-D%C3%BC%C5%9F-r.png"/>
-    <hyperlink ref="C4" r:id="rId3" display="Bilmiş Çocuğun Şarkıları"/>
-    <hyperlink ref="C5" r:id="rId4" display="Bilmiş Çocuğun Şarkıları"/>
-    <hyperlink ref="C6" r:id="rId5" display="Bilmiş Çocuğun Şarkıları"/>
-    <hyperlink ref="C7" r:id="rId6" display="Bilmiş Çocuğun Şarkıları"/>
-    <hyperlink ref="G10" r:id="rId7" display="https://ansiklopedi.subadapcocuk.org/images/thumb/d/d3/Dinonun_%C5%9Fark%C4%B1s%C4%B1_R.png/300px-Dinonun_%C5%9Fark%C4%B1s%C4%B1_R.png?20200628141720"/>
-    <hyperlink ref="E41" r:id="rId8" display="https://ansiklopedi.subadapcocuk.org/index.php/Ne%C5%9Feli_Bir_G%C3%BCn"/>
-    <hyperlink ref="G41" r:id="rId9" display="https://ansiklopedi.subadapcocuk.org/images/thumb/7/73/Ne%C5%9Feli_bi_g%C3%BCn.jpg/300px-Ne%C5%9Feli_bi_g%C3%BCn.jpg"/>
-    <hyperlink ref="E42" r:id="rId10" display="https://ansiklopedi.subadapcocuk.org/index.php/D%C3%BCnyan%C4%B1n_Do%C4%9Fum_G%C3%BCn%C3%BC"/>
-    <hyperlink ref="F42" r:id="rId11" display="https://ansiklopedi.subadapcocuk.org/images/d/d3/D%C3%BCnyan%C4%B1n_do%C4%9Fum_g%C3%BCn%C3%BC.mp3"/>
-    <hyperlink ref="G42" r:id="rId12" display="https://ansiklopedi.subadapcocuk.org/images/thumb/5/5b/D%C3%BCnyan%C4%B1n_do%C4%9Fum_g%C3%BCn%C3%BC_g%C3%B6rsel.jpg/300px-D%C3%BCnyan%C4%B1n_do%C4%9Fum_g%C3%BCn%C3%BC_g%C3%B6rsel.jpg"/>
-    <hyperlink ref="E43" r:id="rId13" display="https://ansiklopedi.subadapcocuk.org/index.php/Okul_Neresi%3F"/>
-    <hyperlink ref="G43" r:id="rId14" display="https://ansiklopedi.subadapcocuk.org/images/thumb/c/c3/Okul_Neresi%3F_G%C3%B6rsel.jpg/300px-Okul_Neresi%3F_G%C3%B6rsel.jpg"/>
-    <hyperlink ref="E44" r:id="rId15" display="https://ansiklopedi.subadapcocuk.org/index.php/En_%C4%B0yisi_De%C4%9Fil!"/>
-    <hyperlink ref="G44" r:id="rId16" display="https://ansiklopedi.subadapcocuk.org/images/thumb/e/e6/En_%C4%B0yisi_De%C4%9Fil.jpg/300px-En_%C4%B0yisi_De%C4%9Fil.jpg"/>
-    <hyperlink ref="E45" r:id="rId17" display="https://ansiklopedi.subadapcocuk.org/index.php/Bir_%C5%9Eiir_Yazd%C4%B1m"/>
-    <hyperlink ref="F45" r:id="rId18" display="https://ansiklopedi.subadapcocuk.org/images/c/ca/Bir_%C5%9Fiir_yazd%C4%B1m.mp3"/>
-    <hyperlink ref="G45" r:id="rId19" display="https://ansiklopedi.subadapcocuk.org/images/thumb/d/d3/Bir_%C5%9Fiir_Yazd%C4%B1m_G%C3%B6rsel.jpg/300px-Bir_%C5%9Fiir_Yazd%C4%B1m_G%C3%B6rsel.jpg"/>
-    <hyperlink ref="E46" r:id="rId20" display="https://ansiklopedi.subadapcocuk.org/index.php/%C3%87ocuk_Halay%C4%B1"/>
-    <hyperlink ref="F46" r:id="rId21" display="https://ansiklopedi.subadapcocuk.org/images/9/96/%C3%87ocuk_halay%C4%B1.mp3"/>
-    <hyperlink ref="G46" r:id="rId22" display="https://ansiklopedi.subadapcocuk.org/images/thumb/4/4d/%C3%87ocuk_halay%C4%B1_g%C3%B6rsel.jpg/300px-%C3%87ocuk_halay%C4%B1_g%C3%B6rsel.jpg"/>
-    <hyperlink ref="E47" r:id="rId23" display="https://ansiklopedi.subadapcocuk.org/index.php/Suzi"/>
-    <hyperlink ref="F47" r:id="rId24" display="https://ansiklopedi.subadapcocuk.org/images/3/31/Suzi.mp3"/>
-    <hyperlink ref="G47" r:id="rId25" display="https://ansiklopedi.subadapcocuk.org/index.php/Dosya:Kabuk_k%C4%B1rma_partisi_alb%C3%BCm_kapa%C4%9F%C4%B1.png"/>
-    <hyperlink ref="E48" r:id="rId26" display="https://ansiklopedi.subadapcocuk.org/index.php/Tak_Tak_Tak"/>
-    <hyperlink ref="F48" r:id="rId27" display="https://ansiklopedi.subadapcocuk.org/images/9/96/Tak_Tak_Tak.mp3"/>
-    <hyperlink ref="G48" r:id="rId28" display="https://ansiklopedi.subadapcocuk.org/index.php/Dosya:Kabuk_k%C4%B1rma_partisi_alb%C3%BCm_kapa%C4%9F%C4%B1.png"/>
-    <hyperlink ref="E49" r:id="rId29" display="https://ansiklopedi.subadapcocuk.org/index.php/%C5%9Ea%C5%9F%C4%B1ran_Mevsimler"/>
-    <hyperlink ref="F49" r:id="rId30" display="https://ansiklopedi.subadapcocuk.org/images/c/c4/%C5%9Ea%C5%9F%C4%B1ran_Mevsimler.mp3"/>
-    <hyperlink ref="G49" r:id="rId31" display="https://ansiklopedi.subadapcocuk.org/index.php/Dosya:Kabuk_k%C4%B1rma_partisi_alb%C3%BCm_kapa%C4%9F%C4%B1.png"/>
-    <hyperlink ref="E50" r:id="rId32" display="https://ansiklopedi.subadapcocuk.org/index.php/Evdeki_Hayalet"/>
-    <hyperlink ref="F50" r:id="rId33" display="https://ansiklopedi.subadapcocuk.org/images/0/0b/Evdeki_Hayalet.mp3"/>
-    <hyperlink ref="G50" r:id="rId34" display="https://ansiklopedi.subadapcocuk.org/index.php/Dosya:Kabuk_k%C4%B1rma_partisi_alb%C3%BCm_kapa%C4%9F%C4%B1.png"/>
-    <hyperlink ref="E51" r:id="rId35" display="https://ansiklopedi.subadapcocuk.org/index.php/Tak%C4%B1l_Kitaplar%C4%B1n_Kanatlar%C4%B1na"/>
-    <hyperlink ref="F51" r:id="rId36" display="https://ansiklopedi.subadapcocuk.org/images/f/f8/Tak%C4%B1l_Kitaplar%C4%B1n_Kanatlar%C4%B1na.mp3"/>
-    <hyperlink ref="G51" r:id="rId37" display="https://ansiklopedi.subadapcocuk.org/index.php/Dosya:Kabuk_k%C4%B1rma_partisi_alb%C3%BCm_kapa%C4%9F%C4%B1.png"/>
-    <hyperlink ref="E52" r:id="rId38" display="https://ansiklopedi.subadapcocuk.org/index.php/%C3%96c%C3%BC_M%C3%B6c%C3%BC_Yok_Ki!"/>
-    <hyperlink ref="F52" r:id="rId39" display="https://ansiklopedi.subadapcocuk.org/images/9/9a/%C3%96c%C3%BC_M%C3%B6c%C3%BC_Yok_Ki.mp3"/>
-    <hyperlink ref="G52" r:id="rId40" display="https://ansiklopedi.subadapcocuk.org/index.php/Dosya:Kabuk_k%C4%B1rma_partisi_alb%C3%BCm_kapa%C4%9F%C4%B1.png"/>
-  </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>